<commit_message>
adjust the fx generator, generalize and test, some smaller fixes and adjustments, use the ensemble ID of the driving model, this is also allowed and more consistent, instead of r0i0p0
</commit_message>
<xml_diff>
--- a/fps_convection_variables_vfinal_2021update_with_addons.xlsx
+++ b/fps_convection_variables_vfinal_2021update_with_addons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kgo/Documents/tools/postpro/WRF_CMORizer_my_dev_with_git/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6C0AE6-2D20-5145-95D2-0131AFAB5822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC2A423-E85C-3D44-AD8F-365B062AE465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10940" yWindow="1240" windowWidth="30460" windowHeight="24000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="880" yWindow="740" windowWidth="26180" windowHeight="17180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core" sheetId="4" r:id="rId1"/>
@@ -2400,7 +2400,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="43">
+  <fonts count="42">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2672,12 +2672,6 @@
       <color theme="1"/>
       <name val="NimbusRomNo9L"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="17">
     <fill>
@@ -5037,6 +5031,119 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="92" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="92" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -5055,6 +5162,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="15" fontId="15" fillId="2" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -5067,126 +5180,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="92" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="92" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5919,7 +5913,7 @@
       <c r="W4" s="28"/>
       <c r="X4" s="28"/>
       <c r="Y4" s="29"/>
-      <c r="Z4" s="270" t="s">
+      <c r="Z4" s="258" t="s">
         <v>7</v>
       </c>
       <c r="AA4" s="134"/>
@@ -5976,7 +5970,7 @@
       <c r="W5" s="43"/>
       <c r="X5" s="43"/>
       <c r="Y5" s="46"/>
-      <c r="Z5" s="270" t="s">
+      <c r="Z5" s="258" t="s">
         <v>7</v>
       </c>
       <c r="AA5" s="135"/>
@@ -6025,14 +6019,14 @@
       </c>
       <c r="R6" s="14"/>
       <c r="S6" s="19"/>
-      <c r="T6" s="308" t="s">
+      <c r="T6" s="296" t="s">
         <v>317</v>
       </c>
       <c r="U6" s="16"/>
       <c r="V6" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W6" s="282" t="s">
+      <c r="W6" s="270" t="s">
         <v>7</v>
       </c>
       <c r="X6" s="25"/>
@@ -6082,14 +6076,14 @@
         <v>111</v>
       </c>
       <c r="S7" s="20"/>
-      <c r="T7" s="308" t="s">
+      <c r="T7" s="296" t="s">
         <v>317</v>
       </c>
       <c r="U7" s="16"/>
       <c r="V7" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W7" s="282" t="s">
+      <c r="W7" s="270" t="s">
         <v>7</v>
       </c>
       <c r="X7" s="28"/>
@@ -6141,14 +6135,14 @@
       </c>
       <c r="R8" s="14"/>
       <c r="S8" s="21"/>
-      <c r="T8" s="304" t="s">
+      <c r="T8" s="292" t="s">
         <v>318</v>
       </c>
       <c r="U8" s="16"/>
       <c r="V8" s="119" t="s">
         <v>115</v>
       </c>
-      <c r="W8" s="279" t="s">
+      <c r="W8" s="267" t="s">
         <v>7</v>
       </c>
       <c r="X8" s="35"/>
@@ -6203,12 +6197,12 @@
       <c r="V9" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W9" s="294" t="s">
+      <c r="W9" s="282" t="s">
         <v>7</v>
       </c>
       <c r="X9" s="16"/>
       <c r="Y9" s="16"/>
-      <c r="Z9" s="295" t="s">
+      <c r="Z9" s="283" t="s">
         <v>7</v>
       </c>
       <c r="AA9" s="141"/>
@@ -6255,7 +6249,7 @@
       </c>
       <c r="R10" s="14"/>
       <c r="S10" s="149"/>
-      <c r="T10" s="301" t="s">
+      <c r="T10" s="289" t="s">
         <v>363</v>
       </c>
       <c r="U10" s="16"/>
@@ -6265,7 +6259,7 @@
       <c r="W10" s="34"/>
       <c r="X10" s="28"/>
       <c r="Y10" s="29"/>
-      <c r="Z10" s="270" t="s">
+      <c r="Z10" s="258" t="s">
         <v>7</v>
       </c>
       <c r="AA10" s="134"/>
@@ -6312,14 +6306,14 @@
       </c>
       <c r="R11" s="14"/>
       <c r="S11" s="20"/>
-      <c r="T11" s="305" t="s">
+      <c r="T11" s="293" t="s">
         <v>317</v>
       </c>
       <c r="U11" s="16"/>
       <c r="V11" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W11" s="282" t="s">
+      <c r="W11" s="270" t="s">
         <v>7</v>
       </c>
       <c r="X11" s="30"/>
@@ -6378,7 +6372,7 @@
       <c r="V12" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W12" s="293" t="s">
+      <c r="W12" s="281" t="s">
         <v>7</v>
       </c>
       <c r="X12" s="30"/>
@@ -6428,15 +6422,15 @@
       </c>
       <c r="R13" s="14"/>
       <c r="S13" s="20"/>
-      <c r="T13" s="300" t="s">
+      <c r="T13" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U13" s="16"/>
       <c r="V13" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W13" s="282"/>
-      <c r="X13" s="275" t="s">
+      <c r="W13" s="270"/>
+      <c r="X13" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y13" s="31"/>
@@ -6485,15 +6479,15 @@
       </c>
       <c r="R14" s="14"/>
       <c r="S14" s="20"/>
-      <c r="T14" s="300" t="s">
+      <c r="T14" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U14" s="16"/>
       <c r="V14" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W14" s="282"/>
-      <c r="X14" s="275" t="s">
+      <c r="W14" s="270"/>
+      <c r="X14" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y14" s="31"/>
@@ -6542,15 +6536,15 @@
       </c>
       <c r="R15" s="14"/>
       <c r="S15" s="20"/>
-      <c r="T15" s="300" t="s">
+      <c r="T15" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U15" s="16"/>
       <c r="V15" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W15" s="282"/>
-      <c r="X15" s="275" t="s">
+      <c r="W15" s="270"/>
+      <c r="X15" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y15" s="31"/>
@@ -6599,15 +6593,15 @@
       </c>
       <c r="R16" s="14"/>
       <c r="S16" s="20"/>
-      <c r="T16" s="300" t="s">
+      <c r="T16" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U16" s="16"/>
       <c r="V16" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W16" s="282"/>
-      <c r="X16" s="275" t="s">
+      <c r="W16" s="270"/>
+      <c r="X16" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y16" s="31"/>
@@ -6656,15 +6650,15 @@
       </c>
       <c r="R17" s="14"/>
       <c r="S17" s="20"/>
-      <c r="T17" s="300" t="s">
+      <c r="T17" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U17" s="16"/>
       <c r="V17" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W17" s="282"/>
-      <c r="X17" s="275" t="s">
+      <c r="W17" s="270"/>
+      <c r="X17" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y17" s="31"/>
@@ -6710,15 +6704,15 @@
       </c>
       <c r="R18" s="14"/>
       <c r="S18" s="20"/>
-      <c r="T18" s="300" t="s">
+      <c r="T18" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U18" s="16"/>
       <c r="V18" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W18" s="282"/>
-      <c r="X18" s="275" t="s">
+      <c r="W18" s="270"/>
+      <c r="X18" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y18" s="31"/>
@@ -6767,14 +6761,14 @@
       </c>
       <c r="R19" s="14"/>
       <c r="S19" s="20"/>
-      <c r="T19" s="305" t="s">
+      <c r="T19" s="293" t="s">
         <v>317</v>
       </c>
       <c r="U19" s="16"/>
       <c r="V19" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W19" s="282" t="s">
+      <c r="W19" s="270" t="s">
         <v>7</v>
       </c>
       <c r="X19" s="30"/>
@@ -6831,7 +6825,7 @@
       <c r="V20" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W20" s="293" t="s">
+      <c r="W20" s="281" t="s">
         <v>7</v>
       </c>
       <c r="X20" s="30"/>
@@ -6881,15 +6875,15 @@
       </c>
       <c r="R21" s="14"/>
       <c r="S21" s="20"/>
-      <c r="T21" s="300" t="s">
+      <c r="T21" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U21" s="16"/>
       <c r="V21" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W21" s="282"/>
-      <c r="X21" s="275" t="s">
+      <c r="W21" s="270"/>
+      <c r="X21" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y21" s="31"/>
@@ -6938,15 +6932,15 @@
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="20"/>
-      <c r="T22" s="300" t="s">
+      <c r="T22" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U22" s="16"/>
       <c r="V22" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W22" s="282"/>
-      <c r="X22" s="275" t="s">
+      <c r="W22" s="270"/>
+      <c r="X22" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y22" s="31"/>
@@ -6995,15 +6989,15 @@
       </c>
       <c r="R23" s="14"/>
       <c r="S23" s="20"/>
-      <c r="T23" s="300" t="s">
+      <c r="T23" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U23" s="16"/>
       <c r="V23" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W23" s="282"/>
-      <c r="X23" s="275" t="s">
+      <c r="W23" s="270"/>
+      <c r="X23" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y23" s="31"/>
@@ -7052,15 +7046,15 @@
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="20"/>
-      <c r="T24" s="300" t="s">
+      <c r="T24" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U24" s="16"/>
       <c r="V24" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W24" s="282"/>
-      <c r="X24" s="275" t="s">
+      <c r="W24" s="270"/>
+      <c r="X24" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y24" s="31"/>
@@ -7109,15 +7103,15 @@
       </c>
       <c r="R25" s="14"/>
       <c r="S25" s="14"/>
-      <c r="T25" s="300" t="s">
+      <c r="T25" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U25" s="16"/>
       <c r="V25" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W25" s="282"/>
-      <c r="X25" s="275" t="s">
+      <c r="W25" s="270"/>
+      <c r="X25" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y25" s="31"/>
@@ -7166,15 +7160,15 @@
       </c>
       <c r="R26" s="14"/>
       <c r="S26" s="14"/>
-      <c r="T26" s="300" t="s">
+      <c r="T26" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U26" s="16"/>
       <c r="V26" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W26" s="282"/>
-      <c r="X26" s="275" t="s">
+      <c r="W26" s="270"/>
+      <c r="X26" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y26" s="31"/>
@@ -7225,15 +7219,15 @@
         <v>373</v>
       </c>
       <c r="S27" s="22"/>
-      <c r="T27" s="300" t="s">
+      <c r="T27" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U27" s="16"/>
       <c r="V27" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W27" s="282"/>
-      <c r="X27" s="275" t="s">
+      <c r="W27" s="270"/>
+      <c r="X27" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y27" s="31"/>
@@ -7284,15 +7278,15 @@
         <v>105</v>
       </c>
       <c r="S28" s="22"/>
-      <c r="T28" s="300" t="s">
+      <c r="T28" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U28" s="16"/>
       <c r="V28" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W28" s="282"/>
-      <c r="X28" s="275" t="s">
+      <c r="W28" s="270"/>
+      <c r="X28" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y28" s="31"/>
@@ -7343,15 +7337,15 @@
         <v>105</v>
       </c>
       <c r="S29" s="22"/>
-      <c r="T29" s="300" t="s">
+      <c r="T29" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U29" s="16"/>
       <c r="V29" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W29" s="282"/>
-      <c r="X29" s="275" t="s">
+      <c r="W29" s="270"/>
+      <c r="X29" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y29" s="31"/>
@@ -7402,15 +7396,15 @@
         <v>105</v>
       </c>
       <c r="S30" s="22"/>
-      <c r="T30" s="300" t="s">
+      <c r="T30" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U30" s="16"/>
       <c r="V30" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W30" s="282"/>
-      <c r="X30" s="275" t="s">
+      <c r="W30" s="270"/>
+      <c r="X30" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y30" s="31"/>
@@ -7461,15 +7455,15 @@
         <v>105</v>
       </c>
       <c r="S31" s="22"/>
-      <c r="T31" s="300" t="s">
+      <c r="T31" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U31" s="16"/>
       <c r="V31" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W31" s="282"/>
-      <c r="X31" s="275" t="s">
+      <c r="W31" s="270"/>
+      <c r="X31" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y31" s="31"/>
@@ -7520,15 +7514,15 @@
         <v>105</v>
       </c>
       <c r="S32" s="22"/>
-      <c r="T32" s="300" t="s">
+      <c r="T32" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U32" s="16"/>
       <c r="V32" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W32" s="282"/>
-      <c r="X32" s="275" t="s">
+      <c r="W32" s="270"/>
+      <c r="X32" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y32" s="31"/>
@@ -7575,17 +7569,17 @@
       </c>
       <c r="R33" s="14"/>
       <c r="S33" s="20"/>
-      <c r="T33" s="305" t="s">
+      <c r="T33" s="293" t="s">
         <v>317</v>
       </c>
       <c r="U33" s="16"/>
       <c r="V33" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W33" s="282" t="s">
+      <c r="W33" s="270" t="s">
         <v>7</v>
       </c>
-      <c r="X33" s="309"/>
+      <c r="X33" s="30"/>
       <c r="Y33" s="31"/>
       <c r="Z33" s="48"/>
       <c r="AA33" s="135"/>
@@ -7633,15 +7627,15 @@
       </c>
       <c r="R34" s="14"/>
       <c r="S34" s="20"/>
-      <c r="T34" s="300" t="s">
+      <c r="T34" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U34" s="16"/>
       <c r="V34" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W34" s="282"/>
-      <c r="X34" s="275" t="s">
+      <c r="W34" s="270"/>
+      <c r="X34" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y34" s="31"/>
@@ -7688,15 +7682,15 @@
       </c>
       <c r="R35" s="14"/>
       <c r="S35" s="20"/>
-      <c r="T35" s="300" t="s">
+      <c r="T35" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U35" s="16"/>
       <c r="V35" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W35" s="282"/>
-      <c r="X35" s="274" t="s">
+      <c r="W35" s="270"/>
+      <c r="X35" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z35" s="48"/>
@@ -7742,15 +7736,15 @@
       </c>
       <c r="R36" s="14"/>
       <c r="S36" s="20"/>
-      <c r="T36" s="300" t="s">
+      <c r="T36" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U36" s="16"/>
       <c r="V36" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W36" s="282"/>
-      <c r="X36" s="275" t="s">
+      <c r="W36" s="270"/>
+      <c r="X36" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y36" s="31"/>
@@ -7797,15 +7791,15 @@
       </c>
       <c r="R37" s="14"/>
       <c r="S37" s="20"/>
-      <c r="T37" s="300" t="s">
+      <c r="T37" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U37" s="16"/>
       <c r="V37" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W37" s="282"/>
-      <c r="X37" s="275" t="s">
+      <c r="W37" s="270"/>
+      <c r="X37" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y37" s="31"/>
@@ -7852,15 +7846,15 @@
       </c>
       <c r="R38" s="14"/>
       <c r="S38" s="20"/>
-      <c r="T38" s="300" t="s">
+      <c r="T38" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U38" s="16"/>
       <c r="V38" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W38" s="282"/>
-      <c r="X38" s="275" t="s">
+      <c r="W38" s="270"/>
+      <c r="X38" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y38" s="31"/>
@@ -7907,15 +7901,15 @@
       </c>
       <c r="R39" s="14"/>
       <c r="S39" s="20"/>
-      <c r="T39" s="300" t="s">
+      <c r="T39" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U39" s="16"/>
       <c r="V39" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W39" s="282"/>
-      <c r="X39" s="275" t="s">
+      <c r="W39" s="270"/>
+      <c r="X39" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y39" s="31"/>
@@ -7962,15 +7956,15 @@
       </c>
       <c r="R40" s="14"/>
       <c r="S40" s="20"/>
-      <c r="T40" s="300" t="s">
+      <c r="T40" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U40" s="16"/>
       <c r="V40" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W40" s="282"/>
-      <c r="X40" s="275" t="s">
+      <c r="W40" s="270"/>
+      <c r="X40" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y40" s="31"/>
@@ -8017,15 +8011,15 @@
       </c>
       <c r="R41" s="14"/>
       <c r="S41" s="20"/>
-      <c r="T41" s="300" t="s">
+      <c r="T41" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U41" s="16"/>
       <c r="V41" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W41" s="282"/>
-      <c r="X41" s="275" t="s">
+      <c r="W41" s="270"/>
+      <c r="X41" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y41" s="31"/>
@@ -8072,15 +8066,15 @@
       </c>
       <c r="R42" s="14"/>
       <c r="S42" s="20"/>
-      <c r="T42" s="300" t="s">
+      <c r="T42" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U42" s="16"/>
       <c r="V42" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W42" s="282"/>
-      <c r="X42" s="275" t="s">
+      <c r="W42" s="270"/>
+      <c r="X42" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y42" s="31"/>
@@ -8127,15 +8121,15 @@
       </c>
       <c r="R43" s="14"/>
       <c r="S43" s="20"/>
-      <c r="T43" s="300" t="s">
+      <c r="T43" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U43" s="16"/>
       <c r="V43" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W43" s="282"/>
-      <c r="X43" s="275" t="s">
+      <c r="W43" s="270"/>
+      <c r="X43" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y43" s="31"/>
@@ -8182,15 +8176,15 @@
       </c>
       <c r="R44" s="14"/>
       <c r="S44" s="20"/>
-      <c r="T44" s="300" t="s">
+      <c r="T44" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U44" s="16"/>
       <c r="V44" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W44" s="282"/>
-      <c r="X44" s="275" t="s">
+      <c r="W44" s="270"/>
+      <c r="X44" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y44" s="31"/>
@@ -8237,15 +8231,15 @@
       </c>
       <c r="R45" s="14"/>
       <c r="S45" s="20"/>
-      <c r="T45" s="300" t="s">
+      <c r="T45" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U45" s="16"/>
       <c r="V45" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W45" s="282"/>
-      <c r="X45" s="275" t="s">
+      <c r="W45" s="270"/>
+      <c r="X45" s="263" t="s">
         <v>7</v>
       </c>
       <c r="Y45" s="31"/>
@@ -8292,16 +8286,16 @@
       </c>
       <c r="R46" s="14"/>
       <c r="S46" s="20"/>
-      <c r="T46" s="300" t="s">
+      <c r="T46" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U46" s="16"/>
       <c r="V46" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W46" s="282"/>
+      <c r="W46" s="270"/>
       <c r="X46" s="30"/>
-      <c r="Y46" s="274" t="s">
+      <c r="Y46" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z46" s="48"/>
@@ -8347,16 +8341,16 @@
       </c>
       <c r="R47" s="14"/>
       <c r="S47" s="20"/>
-      <c r="T47" s="300" t="s">
+      <c r="T47" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U47" s="16"/>
       <c r="V47" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W47" s="282"/>
+      <c r="W47" s="270"/>
       <c r="X47" s="30"/>
-      <c r="Y47" s="274" t="s">
+      <c r="Y47" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z47" s="48"/>
@@ -8402,16 +8396,16 @@
       </c>
       <c r="R48" s="14"/>
       <c r="S48" s="20"/>
-      <c r="T48" s="300" t="s">
+      <c r="T48" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U48" s="16"/>
       <c r="V48" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W48" s="282"/>
+      <c r="W48" s="270"/>
       <c r="X48" s="30"/>
-      <c r="Y48" s="274" t="s">
+      <c r="Y48" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z48" s="48"/>
@@ -8457,16 +8451,16 @@
       </c>
       <c r="R49" s="14"/>
       <c r="S49" s="20"/>
-      <c r="T49" s="300" t="s">
+      <c r="T49" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U49" s="16"/>
       <c r="V49" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W49" s="282"/>
+      <c r="W49" s="270"/>
       <c r="X49" s="30"/>
-      <c r="Y49" s="274" t="s">
+      <c r="Y49" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z49" s="48"/>
@@ -8512,16 +8506,16 @@
       </c>
       <c r="R50" s="14"/>
       <c r="S50" s="20"/>
-      <c r="T50" s="300" t="s">
+      <c r="T50" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U50" s="16"/>
       <c r="V50" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W50" s="282"/>
+      <c r="W50" s="270"/>
       <c r="X50" s="30"/>
-      <c r="Y50" s="274" t="s">
+      <c r="Y50" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z50" s="48"/>
@@ -8567,16 +8561,16 @@
       </c>
       <c r="R51" s="14"/>
       <c r="S51" s="20"/>
-      <c r="T51" s="300" t="s">
+      <c r="T51" s="288" t="s">
         <v>317</v>
       </c>
       <c r="U51" s="16"/>
       <c r="V51" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W51" s="282"/>
+      <c r="W51" s="270"/>
       <c r="X51" s="30"/>
-      <c r="Y51" s="274" t="s">
+      <c r="Y51" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z51" s="48"/>
@@ -8622,16 +8616,16 @@
       </c>
       <c r="R52" s="14"/>
       <c r="S52" s="20"/>
-      <c r="T52" s="305" t="s">
+      <c r="T52" s="293" t="s">
         <v>317</v>
       </c>
       <c r="U52" s="16"/>
       <c r="V52" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W52" s="282"/>
+      <c r="W52" s="270"/>
       <c r="X52" s="30"/>
-      <c r="Y52" s="274" t="s">
+      <c r="Y52" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z52" s="48"/>
@@ -8679,16 +8673,16 @@
         <v>343</v>
       </c>
       <c r="S53" s="20"/>
-      <c r="T53" s="305" t="s">
+      <c r="T53" s="293" t="s">
         <v>317</v>
       </c>
       <c r="U53" s="16"/>
       <c r="V53" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W53" s="282"/>
+      <c r="W53" s="270"/>
       <c r="X53" s="30"/>
-      <c r="Y53" s="274" t="s">
+      <c r="Y53" s="262" t="s">
         <v>7</v>
       </c>
       <c r="Z53" s="48"/>
@@ -8740,14 +8734,14 @@
       <c r="S54" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="T54" s="305" t="s">
+      <c r="T54" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U54" s="16"/>
       <c r="V54" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W54" s="280" t="s">
+      <c r="W54" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X54" s="53"/>
@@ -8801,14 +8795,14 @@
       <c r="S55" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="T55" s="305" t="s">
+      <c r="T55" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U55" s="16"/>
       <c r="V55" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W55" s="280" t="s">
+      <c r="W55" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X55" s="53"/>
@@ -8861,14 +8855,14 @@
       <c r="S56" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="T56" s="305" t="s">
+      <c r="T56" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U56" s="16"/>
       <c r="V56" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W56" s="280" t="s">
+      <c r="W56" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X56" s="53"/>
@@ -8922,14 +8916,14 @@
       <c r="S57" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="T57" s="305" t="s">
+      <c r="T57" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U57" s="16"/>
       <c r="V57" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W57" s="280" t="s">
+      <c r="W57" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X57" s="53"/>
@@ -8983,14 +8977,14 @@
       <c r="S58" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="T58" s="305" t="s">
+      <c r="T58" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U58" s="16"/>
       <c r="V58" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W58" s="280" t="s">
+      <c r="W58" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X58" s="53"/>
@@ -9044,14 +9038,14 @@
       <c r="S59" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="T59" s="305" t="s">
+      <c r="T59" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U59" s="16"/>
       <c r="V59" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W59" s="280" t="s">
+      <c r="W59" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X59" s="53"/>
@@ -9103,14 +9097,14 @@
       </c>
       <c r="R60" s="14"/>
       <c r="S60" s="20"/>
-      <c r="T60" s="305" t="s">
+      <c r="T60" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U60" s="16"/>
       <c r="V60" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W60" s="280" t="s">
+      <c r="W60" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X60" s="53"/>
@@ -9155,14 +9149,14 @@
       </c>
       <c r="R61" s="14"/>
       <c r="S61" s="20"/>
-      <c r="T61" s="305" t="s">
+      <c r="T61" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U61" s="16"/>
       <c r="V61" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W61" s="283" t="s">
+      <c r="W61" s="271" t="s">
         <v>7</v>
       </c>
       <c r="X61" s="53"/>
@@ -9210,14 +9204,14 @@
       </c>
       <c r="R62" s="14"/>
       <c r="S62" s="20"/>
-      <c r="T62" s="305" t="s">
+      <c r="T62" s="293" t="s">
         <v>318</v>
       </c>
       <c r="U62" s="16"/>
       <c r="V62" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="W62" s="280" t="s">
+      <c r="W62" s="268" t="s">
         <v>7</v>
       </c>
       <c r="X62" s="53"/>
@@ -9269,17 +9263,17 @@
         <v>412</v>
       </c>
       <c r="S63" s="20"/>
-      <c r="T63" s="300" t="s">
+      <c r="T63" s="288" t="s">
         <v>318</v>
       </c>
       <c r="U63" s="16"/>
       <c r="V63" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="W63" s="279"/>
+      <c r="W63" s="267"/>
       <c r="X63" s="30"/>
       <c r="Y63" s="31"/>
-      <c r="Z63" s="272" t="s">
+      <c r="Z63" s="260" t="s">
         <v>7</v>
       </c>
       <c r="AA63" s="140"/>
@@ -9330,7 +9324,7 @@
         <v>412</v>
       </c>
       <c r="S64" s="20"/>
-      <c r="T64" s="300" t="s">
+      <c r="T64" s="288" t="s">
         <v>318</v>
       </c>
       <c r="U64" s="20" t="s">
@@ -9339,10 +9333,10 @@
       <c r="V64" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="W64" s="286"/>
+      <c r="W64" s="274"/>
       <c r="X64" s="30"/>
       <c r="Y64" s="31"/>
-      <c r="Z64" s="273" t="s">
+      <c r="Z64" s="261" t="s">
         <v>7</v>
       </c>
       <c r="AA64" s="140"/>
@@ -9390,16 +9384,16 @@
       </c>
       <c r="R65" s="14"/>
       <c r="S65" s="20"/>
-      <c r="T65" s="305" t="s">
+      <c r="T65" s="293" t="s">
         <v>318</v>
       </c>
-      <c r="U65" s="305" t="s">
+      <c r="U65" s="293" t="s">
         <v>121</v>
       </c>
       <c r="V65" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="W65" s="285" t="s">
+      <c r="W65" s="273" t="s">
         <v>7</v>
       </c>
       <c r="X65" s="30"/>
@@ -9450,16 +9444,16 @@
       </c>
       <c r="R66" s="14"/>
       <c r="S66" s="20"/>
-      <c r="T66" s="305" t="s">
+      <c r="T66" s="293" t="s">
         <v>318</v>
       </c>
-      <c r="U66" s="305" t="s">
+      <c r="U66" s="293" t="s">
         <v>121</v>
       </c>
       <c r="V66" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="W66" s="281" t="s">
+      <c r="W66" s="269" t="s">
         <v>7</v>
       </c>
       <c r="X66" s="30"/>
@@ -9516,7 +9510,7 @@
         <v>414</v>
       </c>
       <c r="S67" s="20"/>
-      <c r="T67" s="307" t="s">
+      <c r="T67" s="295" t="s">
         <v>318</v>
       </c>
       <c r="U67" s="20" t="s">
@@ -9525,10 +9519,10 @@
       <c r="V67" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="W67" s="281"/>
+      <c r="W67" s="269"/>
       <c r="X67" s="30"/>
       <c r="Y67" s="31"/>
-      <c r="Z67" s="270" t="s">
+      <c r="Z67" s="258" t="s">
         <v>7</v>
       </c>
       <c r="AA67" s="140"/>
@@ -9581,7 +9575,7 @@
         <v>413</v>
       </c>
       <c r="S68" s="20"/>
-      <c r="T68" s="307" t="s">
+      <c r="T68" s="295" t="s">
         <v>318</v>
       </c>
       <c r="U68" s="20" t="s">
@@ -9590,10 +9584,10 @@
       <c r="V68" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="W68" s="282"/>
+      <c r="W68" s="270"/>
       <c r="X68" s="30"/>
       <c r="Y68" s="31"/>
-      <c r="Z68" s="271" t="s">
+      <c r="Z68" s="259" t="s">
         <v>7</v>
       </c>
       <c r="AA68" s="140"/>
@@ -9638,14 +9632,14 @@
       </c>
       <c r="R69" s="152"/>
       <c r="S69" s="21"/>
-      <c r="T69" s="304" t="s">
+      <c r="T69" s="292" t="s">
         <v>317</v>
       </c>
       <c r="U69" s="16"/>
       <c r="V69" s="153" t="s">
         <v>115</v>
       </c>
-      <c r="W69" s="279" t="s">
+      <c r="W69" s="267" t="s">
         <v>7</v>
       </c>
       <c r="X69" s="35"/>
@@ -9693,14 +9687,14 @@
       </c>
       <c r="R70" s="152"/>
       <c r="S70" s="21"/>
-      <c r="T70" s="304" t="s">
+      <c r="T70" s="292" t="s">
         <v>317</v>
       </c>
       <c r="U70" s="16"/>
       <c r="V70" s="153" t="s">
         <v>115</v>
       </c>
-      <c r="W70" s="279" t="s">
+      <c r="W70" s="267" t="s">
         <v>7</v>
       </c>
       <c r="X70" s="35"/>
@@ -9748,14 +9742,14 @@
       </c>
       <c r="R71" s="152"/>
       <c r="S71" s="21"/>
-      <c r="T71" s="304" t="s">
+      <c r="T71" s="292" t="s">
         <v>317</v>
       </c>
       <c r="U71" s="16"/>
       <c r="V71" s="153" t="s">
         <v>115</v>
       </c>
-      <c r="W71" s="279" t="s">
+      <c r="W71" s="267" t="s">
         <v>7</v>
       </c>
       <c r="X71" s="35"/>
@@ -9787,7 +9781,7 @@
       <c r="M72" s="121"/>
       <c r="N72" s="121"/>
       <c r="O72" s="155"/>
-      <c r="P72" s="156" t="s">
+      <c r="P72" s="309" t="s">
         <v>326</v>
       </c>
       <c r="Q72" s="156" t="s">
@@ -9804,7 +9798,7 @@
       <c r="X72" s="158"/>
       <c r="Y72" s="159"/>
       <c r="Z72" s="160"/>
-      <c r="AA72" s="297" t="s">
+      <c r="AA72" s="285" t="s">
         <v>7</v>
       </c>
     </row>
@@ -9851,7 +9845,7 @@
       <c r="X73" s="158"/>
       <c r="Y73" s="159"/>
       <c r="Z73" s="160"/>
-      <c r="AA73" s="297" t="s">
+      <c r="AA73" s="285" t="s">
         <v>7</v>
       </c>
     </row>
@@ -9896,7 +9890,7 @@
       <c r="X74" s="158"/>
       <c r="Y74" s="159"/>
       <c r="Z74" s="160"/>
-      <c r="AA74" s="298" t="s">
+      <c r="AA74" s="286" t="s">
         <v>7</v>
       </c>
     </row>
@@ -9941,7 +9935,7 @@
       <c r="X75" s="158"/>
       <c r="Y75" s="159"/>
       <c r="Z75" s="160"/>
-      <c r="AA75" s="298" t="s">
+      <c r="AA75" s="286" t="s">
         <v>7</v>
       </c>
     </row>
@@ -9990,7 +9984,7 @@
       <c r="X76" s="158"/>
       <c r="Y76" s="159"/>
       <c r="Z76" s="160"/>
-      <c r="AA76" s="298" t="s">
+      <c r="AA76" s="286" t="s">
         <v>7</v>
       </c>
     </row>
@@ -10037,81 +10031,81 @@
       <c r="X77" s="165"/>
       <c r="Y77" s="172"/>
       <c r="Z77" s="173"/>
-      <c r="AA77" s="299" t="s">
+      <c r="AA77" s="287" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="78" spans="1:32">
-      <c r="A78" s="258" t="s">
+      <c r="A78" s="297" t="s">
         <v>98</v>
       </c>
-      <c r="B78" s="258"/>
-      <c r="C78" s="258"/>
-      <c r="D78" s="258"/>
-      <c r="E78" s="258"/>
-      <c r="F78" s="258"/>
-      <c r="G78" s="258"/>
-      <c r="H78" s="258"/>
-      <c r="I78" s="258"/>
-      <c r="J78" s="258"/>
-      <c r="K78" s="258"/>
-      <c r="L78" s="258"/>
-      <c r="M78" s="258"/>
-      <c r="N78" s="258"/>
-      <c r="O78" s="258"/>
-      <c r="P78" s="258"/>
-      <c r="Q78" s="258"/>
-      <c r="R78" s="258"/>
-      <c r="S78" s="258"/>
-      <c r="T78" s="258"/>
-      <c r="U78" s="258"/>
-      <c r="V78" s="258"/>
-      <c r="W78" s="258"/>
-      <c r="X78" s="258"/>
-      <c r="Y78" s="258"/>
-      <c r="Z78" s="258"/>
-      <c r="AA78" s="258"/>
-      <c r="AB78" s="258"/>
-      <c r="AC78" s="258"/>
-      <c r="AD78" s="258"/>
-      <c r="AE78" s="258"/>
-      <c r="AF78" s="258"/>
+      <c r="B78" s="297"/>
+      <c r="C78" s="297"/>
+      <c r="D78" s="297"/>
+      <c r="E78" s="297"/>
+      <c r="F78" s="297"/>
+      <c r="G78" s="297"/>
+      <c r="H78" s="297"/>
+      <c r="I78" s="297"/>
+      <c r="J78" s="297"/>
+      <c r="K78" s="297"/>
+      <c r="L78" s="297"/>
+      <c r="M78" s="297"/>
+      <c r="N78" s="297"/>
+      <c r="O78" s="297"/>
+      <c r="P78" s="297"/>
+      <c r="Q78" s="297"/>
+      <c r="R78" s="297"/>
+      <c r="S78" s="297"/>
+      <c r="T78" s="297"/>
+      <c r="U78" s="297"/>
+      <c r="V78" s="297"/>
+      <c r="W78" s="297"/>
+      <c r="X78" s="297"/>
+      <c r="Y78" s="297"/>
+      <c r="Z78" s="297"/>
+      <c r="AA78" s="297"/>
+      <c r="AB78" s="297"/>
+      <c r="AC78" s="297"/>
+      <c r="AD78" s="297"/>
+      <c r="AE78" s="297"/>
+      <c r="AF78" s="297"/>
     </row>
     <row r="79" spans="1:32">
-      <c r="A79" s="258" t="s">
+      <c r="A79" s="297" t="s">
         <v>99</v>
       </c>
-      <c r="B79" s="258"/>
-      <c r="C79" s="258"/>
-      <c r="D79" s="258"/>
-      <c r="E79" s="258"/>
-      <c r="F79" s="258"/>
-      <c r="G79" s="258"/>
-      <c r="H79" s="258"/>
-      <c r="I79" s="258"/>
-      <c r="J79" s="258"/>
-      <c r="K79" s="258"/>
-      <c r="L79" s="258"/>
-      <c r="M79" s="258"/>
-      <c r="N79" s="258"/>
-      <c r="O79" s="258"/>
-      <c r="P79" s="258"/>
-      <c r="Q79" s="258"/>
-      <c r="R79" s="258"/>
-      <c r="S79" s="258"/>
-      <c r="T79" s="258"/>
-      <c r="U79" s="258"/>
-      <c r="V79" s="258"/>
-      <c r="W79" s="258"/>
-      <c r="X79" s="258"/>
-      <c r="Y79" s="258"/>
-      <c r="Z79" s="258"/>
-      <c r="AA79" s="258"/>
-      <c r="AB79" s="258"/>
-      <c r="AC79" s="258"/>
-      <c r="AD79" s="258"/>
-      <c r="AE79" s="258"/>
-      <c r="AF79" s="258"/>
+      <c r="B79" s="297"/>
+      <c r="C79" s="297"/>
+      <c r="D79" s="297"/>
+      <c r="E79" s="297"/>
+      <c r="F79" s="297"/>
+      <c r="G79" s="297"/>
+      <c r="H79" s="297"/>
+      <c r="I79" s="297"/>
+      <c r="J79" s="297"/>
+      <c r="K79" s="297"/>
+      <c r="L79" s="297"/>
+      <c r="M79" s="297"/>
+      <c r="N79" s="297"/>
+      <c r="O79" s="297"/>
+      <c r="P79" s="297"/>
+      <c r="Q79" s="297"/>
+      <c r="R79" s="297"/>
+      <c r="S79" s="297"/>
+      <c r="T79" s="297"/>
+      <c r="U79" s="297"/>
+      <c r="V79" s="297"/>
+      <c r="W79" s="297"/>
+      <c r="X79" s="297"/>
+      <c r="Y79" s="297"/>
+      <c r="Z79" s="297"/>
+      <c r="AA79" s="297"/>
+      <c r="AB79" s="297"/>
+      <c r="AC79" s="297"/>
+      <c r="AD79" s="297"/>
+      <c r="AE79" s="297"/>
+      <c r="AF79" s="297"/>
     </row>
     <row r="80" spans="1:32">
       <c r="J80" s="11"/>
@@ -10195,10 +10189,10 @@
       <c r="Q85" s="205" t="s">
         <v>419</v>
       </c>
-      <c r="T85" s="306" t="s">
+      <c r="T85" s="294" t="s">
         <v>318</v>
       </c>
-      <c r="W85" s="284"/>
+      <c r="W85" s="272"/>
     </row>
     <row r="86" spans="1:28" ht="17">
       <c r="A86" s="56">
@@ -10226,10 +10220,10 @@
       <c r="R86" s="222" t="s">
         <v>481</v>
       </c>
-      <c r="T86" s="306" t="s">
+      <c r="T86" s="294" t="s">
         <v>317</v>
       </c>
-      <c r="W86" s="284"/>
+      <c r="W86" s="272"/>
     </row>
     <row r="87" spans="1:28" ht="17">
       <c r="A87" s="56">
@@ -10250,10 +10244,10 @@
       <c r="Q87" s="205" t="s">
         <v>425</v>
       </c>
-      <c r="T87" s="306" t="s">
+      <c r="T87" s="294" t="s">
         <v>318</v>
       </c>
-      <c r="W87" s="284"/>
+      <c r="W87" s="272"/>
     </row>
     <row r="88" spans="1:28" ht="17">
       <c r="A88" s="56">
@@ -10274,10 +10268,10 @@
       <c r="Q88" s="205" t="s">
         <v>424</v>
       </c>
-      <c r="T88" s="306" t="s">
+      <c r="T88" s="294" t="s">
         <v>318</v>
       </c>
-      <c r="W88" s="284"/>
+      <c r="W88" s="272"/>
     </row>
     <row r="89" spans="1:28" ht="17">
       <c r="A89" s="56">
@@ -10300,10 +10294,10 @@
       <c r="Q89" s="205" t="s">
         <v>427</v>
       </c>
-      <c r="T89" s="306" t="s">
+      <c r="T89" s="294" t="s">
         <v>318</v>
       </c>
-      <c r="W89" s="284"/>
+      <c r="W89" s="272"/>
     </row>
     <row r="90" spans="1:28" ht="17">
       <c r="A90" s="56">
@@ -10324,10 +10318,10 @@
       <c r="Q90" s="205" t="s">
         <v>429</v>
       </c>
-      <c r="T90" s="306" t="s">
+      <c r="T90" s="294" t="s">
         <v>392</v>
       </c>
-      <c r="W90" s="284"/>
+      <c r="W90" s="272"/>
     </row>
     <row r="91" spans="1:28" ht="34">
       <c r="A91" s="56">
@@ -10363,7 +10357,7 @@
       <c r="R91" s="222" t="s">
         <v>481</v>
       </c>
-      <c r="W91" s="284"/>
+      <c r="W91" s="272"/>
     </row>
     <row r="92" spans="1:28">
       <c r="A92" s="56">
@@ -10381,10 +10375,10 @@
       <c r="Q92" s="205" t="s">
         <v>433</v>
       </c>
-      <c r="T92" s="306" t="s">
+      <c r="T92" s="294" t="s">
         <v>317</v>
       </c>
-      <c r="W92" s="284"/>
+      <c r="W92" s="272"/>
       <c r="AB92" t="s">
         <v>484</v>
       </c>
@@ -10412,10 +10406,10 @@
       <c r="Q93" s="205" t="s">
         <v>435</v>
       </c>
-      <c r="T93" s="306" t="s">
+      <c r="T93" s="294" t="s">
         <v>318</v>
       </c>
-      <c r="W93" s="284"/>
+      <c r="W93" s="272"/>
     </row>
     <row r="94" spans="1:28" ht="34">
       <c r="A94" s="56">
@@ -10442,10 +10436,10 @@
       <c r="R94" s="222" t="s">
         <v>481</v>
       </c>
-      <c r="T94" s="306" t="s">
+      <c r="T94" s="294" t="s">
         <v>318</v>
       </c>
-      <c r="W94" s="284"/>
+      <c r="W94" s="272"/>
       <c r="AB94" t="s">
         <v>483</v>
       </c>
@@ -10476,10 +10470,10 @@
       <c r="Q95" s="205" t="s">
         <v>349</v>
       </c>
-      <c r="T95" s="306" t="s">
+      <c r="T95" s="294" t="s">
         <v>317</v>
       </c>
-      <c r="W95" s="284"/>
+      <c r="W95" s="272"/>
     </row>
     <row r="96" spans="1:28" ht="17">
       <c r="C96" s="56" t="s">
@@ -10500,7 +10494,7 @@
       <c r="Q96" s="205" t="s">
         <v>449</v>
       </c>
-      <c r="T96" s="306" t="s">
+      <c r="T96" s="294" t="s">
         <v>629</v>
       </c>
     </row>
@@ -10586,10 +10580,10 @@
       <c r="J102" s="202" t="s">
         <v>454</v>
       </c>
-      <c r="T102" s="306" t="s">
+      <c r="T102" s="294" t="s">
         <v>317</v>
       </c>
-      <c r="W102" s="284"/>
+      <c r="W102" s="272"/>
     </row>
     <row r="103" spans="1:23" ht="17">
       <c r="F103" s="56" t="s">
@@ -10601,7 +10595,7 @@
       <c r="J103" s="202" t="s">
         <v>456</v>
       </c>
-      <c r="T103" s="306" t="s">
+      <c r="T103" s="294" t="s">
         <v>318</v>
       </c>
     </row>
@@ -10615,7 +10609,7 @@
       <c r="J104" s="202" t="s">
         <v>457</v>
       </c>
-      <c r="T104" s="306" t="s">
+      <c r="T104" s="294" t="s">
         <v>318</v>
       </c>
     </row>
@@ -10629,7 +10623,7 @@
       <c r="J105" s="202" t="s">
         <v>458</v>
       </c>
-      <c r="T105" s="306" t="s">
+      <c r="T105" s="294" t="s">
         <v>318</v>
       </c>
     </row>
@@ -10646,7 +10640,7 @@
       <c r="J106" s="202" t="s">
         <v>459</v>
       </c>
-      <c r="T106" s="306" t="s">
+      <c r="T106" s="294" t="s">
         <v>317</v>
       </c>
     </row>
@@ -10663,7 +10657,7 @@
       <c r="J107" s="202" t="s">
         <v>460</v>
       </c>
-      <c r="T107" s="306" t="s">
+      <c r="T107" s="294" t="s">
         <v>317</v>
       </c>
     </row>
@@ -10680,7 +10674,7 @@
       <c r="J108" s="202" t="s">
         <v>526</v>
       </c>
-      <c r="T108" s="306" t="s">
+      <c r="T108" s="294" t="s">
         <v>317</v>
       </c>
     </row>
@@ -10697,7 +10691,7 @@
       <c r="J109" s="202" t="s">
         <v>461</v>
       </c>
-      <c r="T109" s="306" t="s">
+      <c r="T109" s="294" t="s">
         <v>317</v>
       </c>
     </row>
@@ -11401,7 +11395,7 @@
       <c r="T4" s="176" t="s">
         <v>115</v>
       </c>
-      <c r="U4" s="287" t="s">
+      <c r="U4" s="275" t="s">
         <v>7</v>
       </c>
       <c r="V4" s="177"/>
@@ -11450,10 +11444,10 @@
       <c r="T5" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="U5" s="292"/>
+      <c r="U5" s="280"/>
       <c r="V5" s="180"/>
       <c r="W5" s="30"/>
-      <c r="X5" s="296" t="s">
+      <c r="X5" s="284" t="s">
         <v>7</v>
       </c>
       <c r="Y5" s="135"/>
@@ -11497,7 +11491,7 @@
       </c>
       <c r="S6" s="183"/>
       <c r="T6" s="121"/>
-      <c r="U6" s="288"/>
+      <c r="U6" s="276"/>
       <c r="V6" s="180"/>
       <c r="W6" s="30"/>
       <c r="X6" s="181" t="s">
@@ -11544,7 +11538,7 @@
       </c>
       <c r="S7" s="183"/>
       <c r="T7" s="121"/>
-      <c r="U7" s="288"/>
+      <c r="U7" s="276"/>
       <c r="V7" s="180"/>
       <c r="W7" s="30"/>
       <c r="X7" s="181" t="s">
@@ -11593,7 +11587,7 @@
       <c r="T8" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="U8" s="289"/>
+      <c r="U8" s="277"/>
       <c r="V8" s="43"/>
       <c r="W8" s="43"/>
       <c r="X8" s="46" t="s">
@@ -11644,7 +11638,7 @@
       <c r="T9" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="U9" s="290" t="s">
+      <c r="U9" s="278" t="s">
         <v>7</v>
       </c>
       <c r="V9" s="190"/>
@@ -11693,7 +11687,7 @@
       </c>
       <c r="S10" s="20"/>
       <c r="T10" s="14"/>
-      <c r="U10" s="291" t="s">
+      <c r="U10" s="279" t="s">
         <v>7</v>
       </c>
       <c r="V10" s="30"/>
@@ -11738,17 +11732,17 @@
         <v>358</v>
       </c>
       <c r="Q11" s="14"/>
-      <c r="R11" s="302" t="s">
+      <c r="R11" s="290" t="s">
         <v>363</v>
       </c>
       <c r="S11" s="20"/>
       <c r="T11" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="U11" s="277"/>
+      <c r="U11" s="265"/>
       <c r="V11" s="30"/>
       <c r="W11" s="31"/>
-      <c r="X11" s="272" t="s">
+      <c r="X11" s="260" t="s">
         <v>7</v>
       </c>
       <c r="Y11" s="136"/>
@@ -11790,88 +11784,88 @@
         <v>357</v>
       </c>
       <c r="Q12" s="168"/>
-      <c r="R12" s="303" t="s">
+      <c r="R12" s="291" t="s">
         <v>363</v>
       </c>
       <c r="S12" s="168"/>
       <c r="T12" s="168" t="s">
         <v>115</v>
       </c>
-      <c r="U12" s="278"/>
+      <c r="U12" s="266"/>
       <c r="V12" s="194"/>
       <c r="W12" s="196"/>
-      <c r="X12" s="276" t="s">
+      <c r="X12" s="264" t="s">
         <v>7</v>
       </c>
       <c r="Y12" s="197"/>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="258" t="s">
+      <c r="A13" s="297" t="s">
         <v>98</v>
       </c>
-      <c r="B13" s="258"/>
-      <c r="C13" s="258"/>
-      <c r="D13" s="258"/>
-      <c r="E13" s="258"/>
-      <c r="F13" s="258"/>
-      <c r="G13" s="258"/>
-      <c r="H13" s="258"/>
-      <c r="I13" s="258"/>
-      <c r="J13" s="258"/>
-      <c r="K13" s="258"/>
-      <c r="L13" s="258"/>
-      <c r="M13" s="258"/>
-      <c r="N13" s="258"/>
-      <c r="O13" s="258"/>
-      <c r="P13" s="258"/>
-      <c r="Q13" s="258"/>
-      <c r="R13" s="258"/>
-      <c r="S13" s="258"/>
-      <c r="T13" s="258"/>
-      <c r="U13" s="258"/>
-      <c r="V13" s="258"/>
-      <c r="W13" s="258"/>
-      <c r="X13" s="258"/>
-      <c r="Y13" s="258"/>
-      <c r="Z13" s="258"/>
-      <c r="AA13" s="258"/>
-      <c r="AB13" s="258"/>
-      <c r="AC13" s="258"/>
-      <c r="AD13" s="258"/>
+      <c r="B13" s="297"/>
+      <c r="C13" s="297"/>
+      <c r="D13" s="297"/>
+      <c r="E13" s="297"/>
+      <c r="F13" s="297"/>
+      <c r="G13" s="297"/>
+      <c r="H13" s="297"/>
+      <c r="I13" s="297"/>
+      <c r="J13" s="297"/>
+      <c r="K13" s="297"/>
+      <c r="L13" s="297"/>
+      <c r="M13" s="297"/>
+      <c r="N13" s="297"/>
+      <c r="O13" s="297"/>
+      <c r="P13" s="297"/>
+      <c r="Q13" s="297"/>
+      <c r="R13" s="297"/>
+      <c r="S13" s="297"/>
+      <c r="T13" s="297"/>
+      <c r="U13" s="297"/>
+      <c r="V13" s="297"/>
+      <c r="W13" s="297"/>
+      <c r="X13" s="297"/>
+      <c r="Y13" s="297"/>
+      <c r="Z13" s="297"/>
+      <c r="AA13" s="297"/>
+      <c r="AB13" s="297"/>
+      <c r="AC13" s="297"/>
+      <c r="AD13" s="297"/>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="258" t="s">
+      <c r="A14" s="297" t="s">
         <v>99</v>
       </c>
-      <c r="B14" s="258"/>
-      <c r="C14" s="258"/>
-      <c r="D14" s="258"/>
-      <c r="E14" s="258"/>
-      <c r="F14" s="258"/>
-      <c r="G14" s="258"/>
-      <c r="H14" s="258"/>
-      <c r="I14" s="258"/>
-      <c r="J14" s="258"/>
-      <c r="K14" s="258"/>
-      <c r="L14" s="258"/>
-      <c r="M14" s="258"/>
-      <c r="N14" s="258"/>
-      <c r="O14" s="258"/>
-      <c r="P14" s="258"/>
-      <c r="Q14" s="258"/>
-      <c r="R14" s="258"/>
-      <c r="S14" s="258"/>
-      <c r="T14" s="258"/>
-      <c r="U14" s="258"/>
-      <c r="V14" s="258"/>
-      <c r="W14" s="258"/>
-      <c r="X14" s="258"/>
-      <c r="Y14" s="258"/>
-      <c r="Z14" s="258"/>
-      <c r="AA14" s="258"/>
-      <c r="AB14" s="258"/>
-      <c r="AC14" s="258"/>
-      <c r="AD14" s="258"/>
+      <c r="B14" s="297"/>
+      <c r="C14" s="297"/>
+      <c r="D14" s="297"/>
+      <c r="E14" s="297"/>
+      <c r="F14" s="297"/>
+      <c r="G14" s="297"/>
+      <c r="H14" s="297"/>
+      <c r="I14" s="297"/>
+      <c r="J14" s="297"/>
+      <c r="K14" s="297"/>
+      <c r="L14" s="297"/>
+      <c r="M14" s="297"/>
+      <c r="N14" s="297"/>
+      <c r="O14" s="297"/>
+      <c r="P14" s="297"/>
+      <c r="Q14" s="297"/>
+      <c r="R14" s="297"/>
+      <c r="S14" s="297"/>
+      <c r="T14" s="297"/>
+      <c r="U14" s="297"/>
+      <c r="V14" s="297"/>
+      <c r="W14" s="297"/>
+      <c r="X14" s="297"/>
+      <c r="Y14" s="297"/>
+      <c r="Z14" s="297"/>
+      <c r="AA14" s="297"/>
+      <c r="AB14" s="297"/>
+      <c r="AC14" s="297"/>
+      <c r="AD14" s="297"/>
     </row>
     <row r="15" spans="1:30">
       <c r="H15" s="11"/>
@@ -11932,12 +11926,12 @@
       <c r="A2" t="s">
         <v>415</v>
       </c>
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="298" t="s">
         <v>149</v>
       </c>
-      <c r="C2" s="259"/>
-      <c r="D2" s="259"/>
-      <c r="E2" s="259"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
       <c r="F2" s="58" t="str">
         <f>[1]all!R5</f>
         <v>10 Feb 2014 Version 3.1</v>
@@ -12415,13 +12409,13 @@
       </c>
     </row>
     <row r="31" spans="2:7" s="60" customFormat="1" ht="36.25" customHeight="1" thickBot="1">
-      <c r="B31" s="259" t="s">
+      <c r="B31" s="298" t="s">
         <v>224</v>
       </c>
-      <c r="C31" s="259"/>
-      <c r="D31" s="259"/>
-      <c r="E31" s="259"/>
-      <c r="F31" s="259"/>
+      <c r="C31" s="298"/>
+      <c r="D31" s="298"/>
+      <c r="E31" s="298"/>
+      <c r="F31" s="298"/>
     </row>
     <row r="32" spans="2:7" s="60" customFormat="1" ht="35" thickBot="1">
       <c r="B32" s="81" t="s">
@@ -12488,13 +12482,13 @@
       <c r="F35" s="80"/>
     </row>
     <row r="36" spans="2:6" s="60" customFormat="1" ht="19" thickBot="1">
-      <c r="B36" s="260" t="s">
+      <c r="B36" s="299" t="s">
         <v>237</v>
       </c>
-      <c r="C36" s="260"/>
-      <c r="D36" s="260"/>
-      <c r="E36" s="260"/>
-      <c r="F36" s="260"/>
+      <c r="C36" s="299"/>
+      <c r="D36" s="299"/>
+      <c r="E36" s="299"/>
+      <c r="F36" s="299"/>
     </row>
     <row r="37" spans="2:6" s="60" customFormat="1" ht="18" thickBot="1">
       <c r="B37" s="81" t="s">
@@ -12618,21 +12612,21 @@
       <c r="E47" s="88"/>
     </row>
     <row r="48" spans="2:6" s="60" customFormat="1">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="300" t="s">
         <v>374</v>
       </c>
-      <c r="C48" s="261"/>
-      <c r="D48" s="261"/>
-      <c r="E48" s="261"/>
+      <c r="C48" s="300"/>
+      <c r="D48" s="300"/>
+      <c r="E48" s="300"/>
     </row>
     <row r="49" spans="2:6" s="60" customFormat="1">
-      <c r="B49" s="262" t="s">
+      <c r="B49" s="301" t="s">
         <v>257</v>
       </c>
-      <c r="C49" s="262"/>
-      <c r="D49" s="262"/>
-      <c r="E49" s="262"/>
-      <c r="F49" s="262"/>
+      <c r="C49" s="301"/>
+      <c r="D49" s="301"/>
+      <c r="E49" s="301"/>
+      <c r="F49" s="301"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -12681,22 +12675,22 @@
       <c r="D2" s="92" t="s">
         <v>259</v>
       </c>
-      <c r="E2" s="264" t="str">
+      <c r="E2" s="305" t="str">
         <f>[1]all!R5</f>
         <v>10 Feb 2014 Version 3.1</v>
       </c>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
-      <c r="P2" s="264"/>
-      <c r="Q2" s="264"/>
+      <c r="F2" s="305"/>
+      <c r="G2" s="305"/>
+      <c r="H2" s="305"/>
+      <c r="I2" s="305"/>
+      <c r="J2" s="305"/>
+      <c r="K2" s="305"/>
+      <c r="L2" s="305"/>
+      <c r="M2" s="305"/>
+      <c r="N2" s="305"/>
+      <c r="O2" s="305"/>
+      <c r="P2" s="305"/>
+      <c r="Q2" s="305"/>
     </row>
     <row r="3" spans="1:17" s="100" customFormat="1">
       <c r="A3" s="93" t="s">
@@ -12709,10 +12703,10 @@
       <c r="D3" s="95" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="265" t="s">
+      <c r="E3" s="306" t="s">
         <v>262</v>
       </c>
-      <c r="F3" s="265"/>
+      <c r="F3" s="306"/>
       <c r="G3" s="96"/>
       <c r="H3" s="96"/>
       <c r="I3" s="96"/>
@@ -12736,13 +12730,13 @@
       <c r="D4" s="104" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="263" t="s">
+      <c r="E4" s="302" t="s">
         <v>263</v>
       </c>
-      <c r="F4" s="263"/>
-      <c r="G4" s="263"/>
-      <c r="H4" s="263"/>
-      <c r="I4" s="263"/>
+      <c r="F4" s="302"/>
+      <c r="G4" s="302"/>
+      <c r="H4" s="302"/>
+      <c r="I4" s="302"/>
       <c r="J4" s="105"/>
       <c r="K4" s="105"/>
       <c r="L4" s="105"/>
@@ -12763,13 +12757,13 @@
       <c r="D5" s="108" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="266" t="s">
+      <c r="E5" s="307" t="s">
         <v>263</v>
       </c>
-      <c r="F5" s="266"/>
-      <c r="G5" s="266"/>
-      <c r="H5" s="266"/>
-      <c r="I5" s="266"/>
+      <c r="F5" s="307"/>
+      <c r="G5" s="307"/>
+      <c r="H5" s="307"/>
+      <c r="I5" s="307"/>
       <c r="J5" s="109"/>
       <c r="K5" s="109"/>
       <c r="L5" s="109"/>
@@ -12813,12 +12807,12 @@
       <c r="K6" s="102" t="s">
         <v>273</v>
       </c>
-      <c r="L6" s="267"/>
-      <c r="M6" s="267"/>
-      <c r="N6" s="267"/>
-      <c r="O6" s="267"/>
-      <c r="P6" s="267"/>
-      <c r="Q6" s="267"/>
+      <c r="L6" s="308"/>
+      <c r="M6" s="308"/>
+      <c r="N6" s="308"/>
+      <c r="O6" s="308"/>
+      <c r="P6" s="308"/>
+      <c r="Q6" s="308"/>
     </row>
     <row r="7" spans="1:17" s="100" customFormat="1" ht="17">
       <c r="A7" s="101" t="s">
@@ -12922,18 +12916,18 @@
       <c r="D10" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E10" s="263" t="s">
+      <c r="E10" s="302" t="s">
         <v>285</v>
       </c>
-      <c r="F10" s="263"/>
-      <c r="G10" s="263"/>
-      <c r="H10" s="263"/>
-      <c r="I10" s="263"/>
-      <c r="J10" s="263"/>
-      <c r="K10" s="263"/>
-      <c r="L10" s="263"/>
-      <c r="M10" s="263"/>
-      <c r="N10" s="263"/>
+      <c r="F10" s="302"/>
+      <c r="G10" s="302"/>
+      <c r="H10" s="302"/>
+      <c r="I10" s="302"/>
+      <c r="J10" s="302"/>
+      <c r="K10" s="302"/>
+      <c r="L10" s="302"/>
+      <c r="M10" s="302"/>
+      <c r="N10" s="302"/>
       <c r="O10" s="105"/>
       <c r="P10" s="105"/>
       <c r="Q10" s="106"/>
@@ -12949,13 +12943,13 @@
       <c r="D11" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E11" s="263" t="s">
+      <c r="E11" s="302" t="s">
         <v>286</v>
       </c>
-      <c r="F11" s="263"/>
-      <c r="G11" s="263"/>
-      <c r="H11" s="263"/>
-      <c r="I11" s="263"/>
+      <c r="F11" s="302"/>
+      <c r="G11" s="302"/>
+      <c r="H11" s="302"/>
+      <c r="I11" s="302"/>
       <c r="J11" s="105"/>
       <c r="K11" s="105"/>
       <c r="L11" s="105"/>
@@ -12982,16 +12976,16 @@
       <c r="F12" s="102" t="s">
         <v>290</v>
       </c>
-      <c r="G12" s="268" t="s">
+      <c r="G12" s="303" t="s">
         <v>291</v>
       </c>
-      <c r="H12" s="268"/>
-      <c r="I12" s="268"/>
-      <c r="J12" s="268"/>
-      <c r="K12" s="268"/>
-      <c r="L12" s="268"/>
-      <c r="M12" s="268"/>
-      <c r="N12" s="268"/>
+      <c r="H12" s="303"/>
+      <c r="I12" s="303"/>
+      <c r="J12" s="303"/>
+      <c r="K12" s="303"/>
+      <c r="L12" s="303"/>
+      <c r="M12" s="303"/>
+      <c r="N12" s="303"/>
       <c r="O12" s="105"/>
       <c r="P12" s="105"/>
       <c r="Q12" s="106"/>
@@ -13007,14 +13001,14 @@
       <c r="D13" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E13" s="263" t="s">
+      <c r="E13" s="302" t="s">
         <v>292</v>
       </c>
-      <c r="F13" s="263"/>
-      <c r="G13" s="263"/>
-      <c r="H13" s="263"/>
-      <c r="I13" s="263"/>
-      <c r="J13" s="263"/>
+      <c r="F13" s="302"/>
+      <c r="G13" s="302"/>
+      <c r="H13" s="302"/>
+      <c r="I13" s="302"/>
+      <c r="J13" s="302"/>
       <c r="K13" s="105"/>
       <c r="L13" s="105"/>
       <c r="M13" s="105"/>
@@ -13143,17 +13137,17 @@
       <c r="D17" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E17" s="263" t="s">
+      <c r="E17" s="302" t="s">
         <v>315</v>
       </c>
-      <c r="F17" s="263"/>
-      <c r="G17" s="263"/>
-      <c r="H17" s="263"/>
-      <c r="I17" s="263"/>
-      <c r="J17" s="263"/>
-      <c r="K17" s="263"/>
-      <c r="L17" s="263"/>
-      <c r="M17" s="263"/>
+      <c r="F17" s="302"/>
+      <c r="G17" s="302"/>
+      <c r="H17" s="302"/>
+      <c r="I17" s="302"/>
+      <c r="J17" s="302"/>
+      <c r="K17" s="302"/>
+      <c r="L17" s="302"/>
+      <c r="M17" s="302"/>
       <c r="N17" s="105"/>
       <c r="O17" s="105"/>
       <c r="P17" s="105"/>
@@ -13170,12 +13164,12 @@
       <c r="D18" s="118" t="s">
         <v>284</v>
       </c>
-      <c r="E18" s="269" t="s">
+      <c r="E18" s="304" t="s">
         <v>316</v>
       </c>
-      <c r="F18" s="269"/>
-      <c r="G18" s="269"/>
-      <c r="H18" s="269"/>
+      <c r="F18" s="304"/>
+      <c r="G18" s="304"/>
+      <c r="H18" s="304"/>
       <c r="I18" s="117"/>
       <c r="J18" s="117"/>
       <c r="K18" s="117"/>
@@ -13193,17 +13187,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="G12:N12"/>
-    <mergeCell ref="E13:J13"/>
-    <mergeCell ref="E17:M17"/>
-    <mergeCell ref="E18:H18"/>
     <mergeCell ref="E10:N10"/>
     <mergeCell ref="E2:Q2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="E4:I4"/>
     <mergeCell ref="E5:I5"/>
     <mergeCell ref="L6:Q6"/>
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="G12:N12"/>
+    <mergeCell ref="E13:J13"/>
+    <mergeCell ref="E17:M17"/>
+    <mergeCell ref="E18:H18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
add sftgif variable as well, testing, fx variables are finished, need geo_em-inputs
</commit_message>
<xml_diff>
--- a/fps_convection_variables_vfinal_2021update_with_addons.xlsx
+++ b/fps_convection_variables_vfinal_2021update_with_addons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kgo/Documents/tools/postpro/WRF_CMORizer_my_dev_with_git/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC2A423-E85C-3D44-AD8F-365B062AE465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24D1197A-8179-E449-8056-FA64ADCC3079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="880" yWindow="740" windowWidth="26180" windowHeight="17180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1340" yWindow="760" windowWidth="48020" windowHeight="17180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core" sheetId="4" r:id="rId1"/>
@@ -5144,6 +5144,9 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -5162,26 +5165,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="15" fontId="15" fillId="2" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="15" fillId="2" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="135">
@@ -5717,20 +5717,17 @@
   <dimension ref="A1:AF158"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="6" width="25" style="56" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="25" style="7" hidden="1" customWidth="1"/>
-    <col min="8" max="9" width="25" style="56" hidden="1" customWidth="1"/>
+    <col min="1" max="6" width="25" style="56" customWidth="1"/>
+    <col min="7" max="7" width="25" style="7" customWidth="1"/>
+    <col min="8" max="9" width="25" style="56" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="13" hidden="1" customWidth="1"/>
+    <col min="11" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1"/>
     <col min="14" max="14" width="11.83203125" customWidth="1"/>
-    <col min="15" max="15" width="10.83203125" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" customWidth="1"/>
     <col min="16" max="16" width="23.6640625" customWidth="1"/>
-    <col min="17" max="17" width="32.1640625" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="23.6640625" hidden="1" customWidth="1"/>
-    <col min="19" max="21" width="23.6640625" customWidth="1"/>
-    <col min="22" max="22" width="23.6640625" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="32.1640625" customWidth="1"/>
+    <col min="18" max="22" width="23.6640625" customWidth="1"/>
     <col min="26" max="27" width="10" style="10" customWidth="1"/>
     <col min="28" max="28" width="18.83203125" customWidth="1"/>
   </cols>
@@ -9781,7 +9778,7 @@
       <c r="M72" s="121"/>
       <c r="N72" s="121"/>
       <c r="O72" s="155"/>
-      <c r="P72" s="309" t="s">
+      <c r="P72" s="297" t="s">
         <v>326</v>
       </c>
       <c r="Q72" s="156" t="s">
@@ -9890,7 +9887,7 @@
       <c r="X74" s="158"/>
       <c r="Y74" s="159"/>
       <c r="Z74" s="160"/>
-      <c r="AA74" s="286" t="s">
+      <c r="AA74" s="285" t="s">
         <v>7</v>
       </c>
     </row>
@@ -9935,7 +9932,7 @@
       <c r="X75" s="158"/>
       <c r="Y75" s="159"/>
       <c r="Z75" s="160"/>
-      <c r="AA75" s="286" t="s">
+      <c r="AA75" s="285" t="s">
         <v>7</v>
       </c>
     </row>
@@ -10036,76 +10033,76 @@
       </c>
     </row>
     <row r="78" spans="1:32">
-      <c r="A78" s="297" t="s">
+      <c r="A78" s="298" t="s">
         <v>98</v>
       </c>
-      <c r="B78" s="297"/>
-      <c r="C78" s="297"/>
-      <c r="D78" s="297"/>
-      <c r="E78" s="297"/>
-      <c r="F78" s="297"/>
-      <c r="G78" s="297"/>
-      <c r="H78" s="297"/>
-      <c r="I78" s="297"/>
-      <c r="J78" s="297"/>
-      <c r="K78" s="297"/>
-      <c r="L78" s="297"/>
-      <c r="M78" s="297"/>
-      <c r="N78" s="297"/>
-      <c r="O78" s="297"/>
-      <c r="P78" s="297"/>
-      <c r="Q78" s="297"/>
-      <c r="R78" s="297"/>
-      <c r="S78" s="297"/>
-      <c r="T78" s="297"/>
-      <c r="U78" s="297"/>
-      <c r="V78" s="297"/>
-      <c r="W78" s="297"/>
-      <c r="X78" s="297"/>
-      <c r="Y78" s="297"/>
-      <c r="Z78" s="297"/>
-      <c r="AA78" s="297"/>
-      <c r="AB78" s="297"/>
-      <c r="AC78" s="297"/>
-      <c r="AD78" s="297"/>
-      <c r="AE78" s="297"/>
-      <c r="AF78" s="297"/>
+      <c r="B78" s="298"/>
+      <c r="C78" s="298"/>
+      <c r="D78" s="298"/>
+      <c r="E78" s="298"/>
+      <c r="F78" s="298"/>
+      <c r="G78" s="298"/>
+      <c r="H78" s="298"/>
+      <c r="I78" s="298"/>
+      <c r="J78" s="298"/>
+      <c r="K78" s="298"/>
+      <c r="L78" s="298"/>
+      <c r="M78" s="298"/>
+      <c r="N78" s="298"/>
+      <c r="O78" s="298"/>
+      <c r="P78" s="298"/>
+      <c r="Q78" s="298"/>
+      <c r="R78" s="298"/>
+      <c r="S78" s="298"/>
+      <c r="T78" s="298"/>
+      <c r="U78" s="298"/>
+      <c r="V78" s="298"/>
+      <c r="W78" s="298"/>
+      <c r="X78" s="298"/>
+      <c r="Y78" s="298"/>
+      <c r="Z78" s="298"/>
+      <c r="AA78" s="298"/>
+      <c r="AB78" s="298"/>
+      <c r="AC78" s="298"/>
+      <c r="AD78" s="298"/>
+      <c r="AE78" s="298"/>
+      <c r="AF78" s="298"/>
     </row>
     <row r="79" spans="1:32">
-      <c r="A79" s="297" t="s">
+      <c r="A79" s="298" t="s">
         <v>99</v>
       </c>
-      <c r="B79" s="297"/>
-      <c r="C79" s="297"/>
-      <c r="D79" s="297"/>
-      <c r="E79" s="297"/>
-      <c r="F79" s="297"/>
-      <c r="G79" s="297"/>
-      <c r="H79" s="297"/>
-      <c r="I79" s="297"/>
-      <c r="J79" s="297"/>
-      <c r="K79" s="297"/>
-      <c r="L79" s="297"/>
-      <c r="M79" s="297"/>
-      <c r="N79" s="297"/>
-      <c r="O79" s="297"/>
-      <c r="P79" s="297"/>
-      <c r="Q79" s="297"/>
-      <c r="R79" s="297"/>
-      <c r="S79" s="297"/>
-      <c r="T79" s="297"/>
-      <c r="U79" s="297"/>
-      <c r="V79" s="297"/>
-      <c r="W79" s="297"/>
-      <c r="X79" s="297"/>
-      <c r="Y79" s="297"/>
-      <c r="Z79" s="297"/>
-      <c r="AA79" s="297"/>
-      <c r="AB79" s="297"/>
-      <c r="AC79" s="297"/>
-      <c r="AD79" s="297"/>
-      <c r="AE79" s="297"/>
-      <c r="AF79" s="297"/>
+      <c r="B79" s="298"/>
+      <c r="C79" s="298"/>
+      <c r="D79" s="298"/>
+      <c r="E79" s="298"/>
+      <c r="F79" s="298"/>
+      <c r="G79" s="298"/>
+      <c r="H79" s="298"/>
+      <c r="I79" s="298"/>
+      <c r="J79" s="298"/>
+      <c r="K79" s="298"/>
+      <c r="L79" s="298"/>
+      <c r="M79" s="298"/>
+      <c r="N79" s="298"/>
+      <c r="O79" s="298"/>
+      <c r="P79" s="298"/>
+      <c r="Q79" s="298"/>
+      <c r="R79" s="298"/>
+      <c r="S79" s="298"/>
+      <c r="T79" s="298"/>
+      <c r="U79" s="298"/>
+      <c r="V79" s="298"/>
+      <c r="W79" s="298"/>
+      <c r="X79" s="298"/>
+      <c r="Y79" s="298"/>
+      <c r="Z79" s="298"/>
+      <c r="AA79" s="298"/>
+      <c r="AB79" s="298"/>
+      <c r="AC79" s="298"/>
+      <c r="AD79" s="298"/>
+      <c r="AE79" s="298"/>
+      <c r="AF79" s="298"/>
     </row>
     <row r="80" spans="1:32">
       <c r="J80" s="11"/>
@@ -11800,72 +11797,72 @@
       <c r="Y12" s="197"/>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="297" t="s">
+      <c r="A13" s="298" t="s">
         <v>98</v>
       </c>
-      <c r="B13" s="297"/>
-      <c r="C13" s="297"/>
-      <c r="D13" s="297"/>
-      <c r="E13" s="297"/>
-      <c r="F13" s="297"/>
-      <c r="G13" s="297"/>
-      <c r="H13" s="297"/>
-      <c r="I13" s="297"/>
-      <c r="J13" s="297"/>
-      <c r="K13" s="297"/>
-      <c r="L13" s="297"/>
-      <c r="M13" s="297"/>
-      <c r="N13" s="297"/>
-      <c r="O13" s="297"/>
-      <c r="P13" s="297"/>
-      <c r="Q13" s="297"/>
-      <c r="R13" s="297"/>
-      <c r="S13" s="297"/>
-      <c r="T13" s="297"/>
-      <c r="U13" s="297"/>
-      <c r="V13" s="297"/>
-      <c r="W13" s="297"/>
-      <c r="X13" s="297"/>
-      <c r="Y13" s="297"/>
-      <c r="Z13" s="297"/>
-      <c r="AA13" s="297"/>
-      <c r="AB13" s="297"/>
-      <c r="AC13" s="297"/>
-      <c r="AD13" s="297"/>
+      <c r="B13" s="298"/>
+      <c r="C13" s="298"/>
+      <c r="D13" s="298"/>
+      <c r="E13" s="298"/>
+      <c r="F13" s="298"/>
+      <c r="G13" s="298"/>
+      <c r="H13" s="298"/>
+      <c r="I13" s="298"/>
+      <c r="J13" s="298"/>
+      <c r="K13" s="298"/>
+      <c r="L13" s="298"/>
+      <c r="M13" s="298"/>
+      <c r="N13" s="298"/>
+      <c r="O13" s="298"/>
+      <c r="P13" s="298"/>
+      <c r="Q13" s="298"/>
+      <c r="R13" s="298"/>
+      <c r="S13" s="298"/>
+      <c r="T13" s="298"/>
+      <c r="U13" s="298"/>
+      <c r="V13" s="298"/>
+      <c r="W13" s="298"/>
+      <c r="X13" s="298"/>
+      <c r="Y13" s="298"/>
+      <c r="Z13" s="298"/>
+      <c r="AA13" s="298"/>
+      <c r="AB13" s="298"/>
+      <c r="AC13" s="298"/>
+      <c r="AD13" s="298"/>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="297" t="s">
+      <c r="A14" s="298" t="s">
         <v>99</v>
       </c>
-      <c r="B14" s="297"/>
-      <c r="C14" s="297"/>
-      <c r="D14" s="297"/>
-      <c r="E14" s="297"/>
-      <c r="F14" s="297"/>
-      <c r="G14" s="297"/>
-      <c r="H14" s="297"/>
-      <c r="I14" s="297"/>
-      <c r="J14" s="297"/>
-      <c r="K14" s="297"/>
-      <c r="L14" s="297"/>
-      <c r="M14" s="297"/>
-      <c r="N14" s="297"/>
-      <c r="O14" s="297"/>
-      <c r="P14" s="297"/>
-      <c r="Q14" s="297"/>
-      <c r="R14" s="297"/>
-      <c r="S14" s="297"/>
-      <c r="T14" s="297"/>
-      <c r="U14" s="297"/>
-      <c r="V14" s="297"/>
-      <c r="W14" s="297"/>
-      <c r="X14" s="297"/>
-      <c r="Y14" s="297"/>
-      <c r="Z14" s="297"/>
-      <c r="AA14" s="297"/>
-      <c r="AB14" s="297"/>
-      <c r="AC14" s="297"/>
-      <c r="AD14" s="297"/>
+      <c r="B14" s="298"/>
+      <c r="C14" s="298"/>
+      <c r="D14" s="298"/>
+      <c r="E14" s="298"/>
+      <c r="F14" s="298"/>
+      <c r="G14" s="298"/>
+      <c r="H14" s="298"/>
+      <c r="I14" s="298"/>
+      <c r="J14" s="298"/>
+      <c r="K14" s="298"/>
+      <c r="L14" s="298"/>
+      <c r="M14" s="298"/>
+      <c r="N14" s="298"/>
+      <c r="O14" s="298"/>
+      <c r="P14" s="298"/>
+      <c r="Q14" s="298"/>
+      <c r="R14" s="298"/>
+      <c r="S14" s="298"/>
+      <c r="T14" s="298"/>
+      <c r="U14" s="298"/>
+      <c r="V14" s="298"/>
+      <c r="W14" s="298"/>
+      <c r="X14" s="298"/>
+      <c r="Y14" s="298"/>
+      <c r="Z14" s="298"/>
+      <c r="AA14" s="298"/>
+      <c r="AB14" s="298"/>
+      <c r="AC14" s="298"/>
+      <c r="AD14" s="298"/>
     </row>
     <row r="15" spans="1:30">
       <c r="H15" s="11"/>
@@ -11926,12 +11923,12 @@
       <c r="A2" t="s">
         <v>415</v>
       </c>
-      <c r="B2" s="298" t="s">
+      <c r="B2" s="299" t="s">
         <v>149</v>
       </c>
-      <c r="C2" s="298"/>
-      <c r="D2" s="298"/>
-      <c r="E2" s="298"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
       <c r="F2" s="58" t="str">
         <f>[1]all!R5</f>
         <v>10 Feb 2014 Version 3.1</v>
@@ -12409,13 +12406,13 @@
       </c>
     </row>
     <row r="31" spans="2:7" s="60" customFormat="1" ht="36.25" customHeight="1" thickBot="1">
-      <c r="B31" s="298" t="s">
+      <c r="B31" s="299" t="s">
         <v>224</v>
       </c>
-      <c r="C31" s="298"/>
-      <c r="D31" s="298"/>
-      <c r="E31" s="298"/>
-      <c r="F31" s="298"/>
+      <c r="C31" s="299"/>
+      <c r="D31" s="299"/>
+      <c r="E31" s="299"/>
+      <c r="F31" s="299"/>
     </row>
     <row r="32" spans="2:7" s="60" customFormat="1" ht="35" thickBot="1">
       <c r="B32" s="81" t="s">
@@ -12482,13 +12479,13 @@
       <c r="F35" s="80"/>
     </row>
     <row r="36" spans="2:6" s="60" customFormat="1" ht="19" thickBot="1">
-      <c r="B36" s="299" t="s">
+      <c r="B36" s="300" t="s">
         <v>237</v>
       </c>
-      <c r="C36" s="299"/>
-      <c r="D36" s="299"/>
-      <c r="E36" s="299"/>
-      <c r="F36" s="299"/>
+      <c r="C36" s="300"/>
+      <c r="D36" s="300"/>
+      <c r="E36" s="300"/>
+      <c r="F36" s="300"/>
     </row>
     <row r="37" spans="2:6" s="60" customFormat="1" ht="18" thickBot="1">
       <c r="B37" s="81" t="s">
@@ -12612,21 +12609,21 @@
       <c r="E47" s="88"/>
     </row>
     <row r="48" spans="2:6" s="60" customFormat="1">
-      <c r="B48" s="300" t="s">
+      <c r="B48" s="301" t="s">
         <v>374</v>
       </c>
-      <c r="C48" s="300"/>
-      <c r="D48" s="300"/>
-      <c r="E48" s="300"/>
+      <c r="C48" s="301"/>
+      <c r="D48" s="301"/>
+      <c r="E48" s="301"/>
     </row>
     <row r="49" spans="2:6" s="60" customFormat="1">
-      <c r="B49" s="301" t="s">
+      <c r="B49" s="302" t="s">
         <v>257</v>
       </c>
-      <c r="C49" s="301"/>
-      <c r="D49" s="301"/>
-      <c r="E49" s="301"/>
-      <c r="F49" s="301"/>
+      <c r="C49" s="302"/>
+      <c r="D49" s="302"/>
+      <c r="E49" s="302"/>
+      <c r="F49" s="302"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -12675,22 +12672,22 @@
       <c r="D2" s="92" t="s">
         <v>259</v>
       </c>
-      <c r="E2" s="305" t="str">
+      <c r="E2" s="304" t="str">
         <f>[1]all!R5</f>
         <v>10 Feb 2014 Version 3.1</v>
       </c>
-      <c r="F2" s="305"/>
-      <c r="G2" s="305"/>
-      <c r="H2" s="305"/>
-      <c r="I2" s="305"/>
-      <c r="J2" s="305"/>
-      <c r="K2" s="305"/>
-      <c r="L2" s="305"/>
-      <c r="M2" s="305"/>
-      <c r="N2" s="305"/>
-      <c r="O2" s="305"/>
-      <c r="P2" s="305"/>
-      <c r="Q2" s="305"/>
+      <c r="F2" s="304"/>
+      <c r="G2" s="304"/>
+      <c r="H2" s="304"/>
+      <c r="I2" s="304"/>
+      <c r="J2" s="304"/>
+      <c r="K2" s="304"/>
+      <c r="L2" s="304"/>
+      <c r="M2" s="304"/>
+      <c r="N2" s="304"/>
+      <c r="O2" s="304"/>
+      <c r="P2" s="304"/>
+      <c r="Q2" s="304"/>
     </row>
     <row r="3" spans="1:17" s="100" customFormat="1">
       <c r="A3" s="93" t="s">
@@ -12703,10 +12700,10 @@
       <c r="D3" s="95" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="306" t="s">
+      <c r="E3" s="305" t="s">
         <v>262</v>
       </c>
-      <c r="F3" s="306"/>
+      <c r="F3" s="305"/>
       <c r="G3" s="96"/>
       <c r="H3" s="96"/>
       <c r="I3" s="96"/>
@@ -12730,13 +12727,13 @@
       <c r="D4" s="104" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="302" t="s">
+      <c r="E4" s="303" t="s">
         <v>263</v>
       </c>
-      <c r="F4" s="302"/>
-      <c r="G4" s="302"/>
-      <c r="H4" s="302"/>
-      <c r="I4" s="302"/>
+      <c r="F4" s="303"/>
+      <c r="G4" s="303"/>
+      <c r="H4" s="303"/>
+      <c r="I4" s="303"/>
       <c r="J4" s="105"/>
       <c r="K4" s="105"/>
       <c r="L4" s="105"/>
@@ -12757,13 +12754,13 @@
       <c r="D5" s="108" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="307" t="s">
+      <c r="E5" s="306" t="s">
         <v>263</v>
       </c>
-      <c r="F5" s="307"/>
-      <c r="G5" s="307"/>
-      <c r="H5" s="307"/>
-      <c r="I5" s="307"/>
+      <c r="F5" s="306"/>
+      <c r="G5" s="306"/>
+      <c r="H5" s="306"/>
+      <c r="I5" s="306"/>
       <c r="J5" s="109"/>
       <c r="K5" s="109"/>
       <c r="L5" s="109"/>
@@ -12807,12 +12804,12 @@
       <c r="K6" s="102" t="s">
         <v>273</v>
       </c>
-      <c r="L6" s="308"/>
-      <c r="M6" s="308"/>
-      <c r="N6" s="308"/>
-      <c r="O6" s="308"/>
-      <c r="P6" s="308"/>
-      <c r="Q6" s="308"/>
+      <c r="L6" s="307"/>
+      <c r="M6" s="307"/>
+      <c r="N6" s="307"/>
+      <c r="O6" s="307"/>
+      <c r="P6" s="307"/>
+      <c r="Q6" s="307"/>
     </row>
     <row r="7" spans="1:17" s="100" customFormat="1" ht="17">
       <c r="A7" s="101" t="s">
@@ -12916,18 +12913,18 @@
       <c r="D10" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E10" s="302" t="s">
+      <c r="E10" s="303" t="s">
         <v>285</v>
       </c>
-      <c r="F10" s="302"/>
-      <c r="G10" s="302"/>
-      <c r="H10" s="302"/>
-      <c r="I10" s="302"/>
-      <c r="J10" s="302"/>
-      <c r="K10" s="302"/>
-      <c r="L10" s="302"/>
-      <c r="M10" s="302"/>
-      <c r="N10" s="302"/>
+      <c r="F10" s="303"/>
+      <c r="G10" s="303"/>
+      <c r="H10" s="303"/>
+      <c r="I10" s="303"/>
+      <c r="J10" s="303"/>
+      <c r="K10" s="303"/>
+      <c r="L10" s="303"/>
+      <c r="M10" s="303"/>
+      <c r="N10" s="303"/>
       <c r="O10" s="105"/>
       <c r="P10" s="105"/>
       <c r="Q10" s="106"/>
@@ -12943,13 +12940,13 @@
       <c r="D11" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E11" s="302" t="s">
+      <c r="E11" s="303" t="s">
         <v>286</v>
       </c>
-      <c r="F11" s="302"/>
-      <c r="G11" s="302"/>
-      <c r="H11" s="302"/>
-      <c r="I11" s="302"/>
+      <c r="F11" s="303"/>
+      <c r="G11" s="303"/>
+      <c r="H11" s="303"/>
+      <c r="I11" s="303"/>
       <c r="J11" s="105"/>
       <c r="K11" s="105"/>
       <c r="L11" s="105"/>
@@ -12976,16 +12973,16 @@
       <c r="F12" s="102" t="s">
         <v>290</v>
       </c>
-      <c r="G12" s="303" t="s">
+      <c r="G12" s="308" t="s">
         <v>291</v>
       </c>
-      <c r="H12" s="303"/>
-      <c r="I12" s="303"/>
-      <c r="J12" s="303"/>
-      <c r="K12" s="303"/>
-      <c r="L12" s="303"/>
-      <c r="M12" s="303"/>
-      <c r="N12" s="303"/>
+      <c r="H12" s="308"/>
+      <c r="I12" s="308"/>
+      <c r="J12" s="308"/>
+      <c r="K12" s="308"/>
+      <c r="L12" s="308"/>
+      <c r="M12" s="308"/>
+      <c r="N12" s="308"/>
       <c r="O12" s="105"/>
       <c r="P12" s="105"/>
       <c r="Q12" s="106"/>
@@ -13001,14 +12998,14 @@
       <c r="D13" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E13" s="302" t="s">
+      <c r="E13" s="303" t="s">
         <v>292</v>
       </c>
-      <c r="F13" s="302"/>
-      <c r="G13" s="302"/>
-      <c r="H13" s="302"/>
-      <c r="I13" s="302"/>
-      <c r="J13" s="302"/>
+      <c r="F13" s="303"/>
+      <c r="G13" s="303"/>
+      <c r="H13" s="303"/>
+      <c r="I13" s="303"/>
+      <c r="J13" s="303"/>
       <c r="K13" s="105"/>
       <c r="L13" s="105"/>
       <c r="M13" s="105"/>
@@ -13137,17 +13134,17 @@
       <c r="D17" s="108" t="s">
         <v>284</v>
       </c>
-      <c r="E17" s="302" t="s">
+      <c r="E17" s="303" t="s">
         <v>315</v>
       </c>
-      <c r="F17" s="302"/>
-      <c r="G17" s="302"/>
-      <c r="H17" s="302"/>
-      <c r="I17" s="302"/>
-      <c r="J17" s="302"/>
-      <c r="K17" s="302"/>
-      <c r="L17" s="302"/>
-      <c r="M17" s="302"/>
+      <c r="F17" s="303"/>
+      <c r="G17" s="303"/>
+      <c r="H17" s="303"/>
+      <c r="I17" s="303"/>
+      <c r="J17" s="303"/>
+      <c r="K17" s="303"/>
+      <c r="L17" s="303"/>
+      <c r="M17" s="303"/>
       <c r="N17" s="105"/>
       <c r="O17" s="105"/>
       <c r="P17" s="105"/>
@@ -13164,12 +13161,12 @@
       <c r="D18" s="118" t="s">
         <v>284</v>
       </c>
-      <c r="E18" s="304" t="s">
+      <c r="E18" s="309" t="s">
         <v>316</v>
       </c>
-      <c r="F18" s="304"/>
-      <c r="G18" s="304"/>
-      <c r="H18" s="304"/>
+      <c r="F18" s="309"/>
+      <c r="G18" s="309"/>
+      <c r="H18" s="309"/>
       <c r="I18" s="117"/>
       <c r="J18" s="117"/>
       <c r="K18" s="117"/>
@@ -13187,17 +13184,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="G12:N12"/>
+    <mergeCell ref="E13:J13"/>
+    <mergeCell ref="E17:M17"/>
+    <mergeCell ref="E18:H18"/>
     <mergeCell ref="E10:N10"/>
     <mergeCell ref="E2:Q2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="E4:I4"/>
     <mergeCell ref="E5:I5"/>
     <mergeCell ref="L6:Q6"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="G12:N12"/>
-    <mergeCell ref="E13:J13"/>
-    <mergeCell ref="E17:M17"/>
-    <mergeCell ref="E18:H18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>